<commit_message>
feat(bonds): Add several tests on portfolio creation and asset generation + new fontend visualization
</commit_message>
<xml_diff>
--- a/data/Assets.xlsx
+++ b/data/Assets.xlsx
@@ -10,9 +10,9 @@
   <sheets>
     <sheet name="Stocks" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Mappings" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Bonds" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="BondsDividends" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="IntDiv" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Summary" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Bonds" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Stocks!$A$1:$H$23</definedName>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="54">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -35,39 +35,42 @@
     <t xml:space="preserve">Ticker</t>
   </si>
   <si>
+    <t xml:space="preserve">Asset Type</t>
+  </si>
+  <si>
     <t xml:space="preserve">Quantity</t>
   </si>
   <si>
     <t xml:space="preserve">Price</t>
   </si>
   <si>
-    <t xml:space="preserve">CalculatedQuantity</t>
-  </si>
-  <si>
     <t xml:space="preserve">Currency</t>
   </si>
   <si>
     <t xml:space="preserve">Investment</t>
   </si>
   <si>
-    <t xml:space="preserve">AssetName</t>
+    <t xml:space="preserve">Asset Name</t>
   </si>
   <si>
     <t xml:space="preserve">CSSPX.MI</t>
   </si>
   <si>
+    <t xml:space="preserve">Stock</t>
+  </si>
+  <si>
     <t xml:space="preserve">EUR</t>
   </si>
   <si>
-    <t xml:space="preserve">TotalAssets</t>
-  </si>
-  <si>
     <t xml:space="preserve">EUNL.DE</t>
   </si>
   <si>
     <t xml:space="preserve">APC.DE</t>
   </si>
   <si>
+    <t xml:space="preserve">ETF</t>
+  </si>
+  <si>
     <t xml:space="preserve">XEON.DE</t>
   </si>
   <si>
@@ -86,9 +89,6 @@
     <t xml:space="preserve">1GOOGL.MI</t>
   </si>
   <si>
-    <t xml:space="preserve">Asset Name</t>
-  </si>
-  <si>
     <t xml:space="preserve">Google</t>
   </si>
   <si>
@@ -140,9 +140,6 @@
     <t xml:space="preserve">TR</t>
   </si>
   <si>
-    <t xml:space="preserve">Total Dividends</t>
-  </si>
-  <si>
     <t xml:space="preserve">Euro Swap</t>
   </si>
   <si>
@@ -152,13 +149,13 @@
     <t xml:space="preserve">Name</t>
   </si>
   <si>
-    <t xml:space="preserve">BondType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Expiry</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FaceValue</t>
+    <t xml:space="preserve">Bond Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maturity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Face Value</t>
   </si>
   <si>
     <t xml:space="preserve">Invested</t>
@@ -170,16 +167,13 @@
     <t xml:space="preserve">IT0005530032</t>
   </si>
   <si>
-    <t xml:space="preserve">Italy 2</t>
+    <t xml:space="preserve">Italy</t>
   </si>
   <si>
     <t xml:space="preserve">Government</t>
   </si>
   <si>
     <t xml:space="preserve">IT0005340929</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italy</t>
   </si>
   <si>
     <t xml:space="preserve">XS2282095970</t>
@@ -516,13 +510,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="9.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="5.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="47.59"/>
@@ -562,11 +555,14 @@
       <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>0.3257696</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>200</v>
@@ -575,9 +571,6 @@
         <f aca="false">_xlfn.XLOOKUP(B2,Mappings!$A$2:$A$10,Mappings!$B$2:$B$10)</f>
         <v>Google</v>
       </c>
-      <c r="J2" s="1" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
@@ -586,11 +579,14 @@
       <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="n">
+      <c r="C3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="n">
         <v>1.889287</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>200</v>
@@ -599,10 +595,6 @@
         <f aca="false">_xlfn.XLOOKUP(B3,Mappings!$A$2:$A$10,Mappings!$B$2:$B$10)</f>
         <v>Nasdaq</v>
       </c>
-      <c r="J3" s="1" t="n">
-        <f aca="false">SUM($G$2:G1000)</f>
-        <v>6250.3</v>
-      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
@@ -611,11 +603,14 @@
       <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1" t="n">
         <v>0.844772</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>200</v>
@@ -630,13 +625,16 @@
         <v>45686</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="n">
+      <c r="D5" s="1" t="n">
         <v>3.927853</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>500</v>
@@ -651,13 +649,16 @@
         <v>45686</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="n">
         <v>3.927853</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>500</v>
@@ -674,11 +675,14 @@
       <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="2" t="n">
+      <c r="C7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>0.811661</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G7" s="1" t="n">
         <v>500</v>
@@ -693,13 +697,16 @@
         <v>45691</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1" t="n">
         <v>3.631873</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G8" s="1" t="n">
         <v>500</v>
@@ -714,13 +721,16 @@
         <v>45705</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="1" t="n">
         <v>1.576789</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G9" s="1" t="n">
         <v>100</v>
@@ -737,11 +747,14 @@
       <c r="B10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="2" t="n">
+      <c r="C10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="n">
         <v>0.82949</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>500</v>
@@ -756,13 +769,16 @@
         <v>45733</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="1" t="n">
         <v>1.620745</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G11" s="1" t="n">
         <v>100</v>
@@ -779,11 +795,14 @@
       <c r="B12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="2" t="n">
+      <c r="C12" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2" t="n">
         <v>0.907803</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G12" s="1" t="n">
         <v>500</v>
@@ -798,13 +817,16 @@
         <v>45751</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2" t="n">
         <v>15.243902</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G13" s="1" t="n">
         <v>1000.3</v>
@@ -819,13 +841,16 @@
         <v>45763</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1" t="n">
         <v>1.717327</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G14" s="1" t="n">
         <v>100</v>
@@ -840,16 +865,19 @@
         <v>45763</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="1" t="n">
         <v>1.576292</v>
       </c>
-      <c r="D15" s="1" t="n">
+      <c r="E15" s="1" t="n">
         <v>63.65</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G15" s="1" t="n">
         <v>100</v>
@@ -864,13 +892,16 @@
         <v>45779</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="2" t="n">
         <v>0.346308</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G16" s="1" t="n">
         <v>50</v>
@@ -885,13 +916,16 @@
         <v>45779</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="2" t="n">
         <v>0.73303</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G17" s="1" t="n">
         <v>50</v>
@@ -908,11 +942,14 @@
       <c r="B18" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C18" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>0.94568</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G18" s="1" t="n">
         <v>500</v>
@@ -927,13 +964,16 @@
         <v>45779</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="1" t="n">
         <v>4.032908</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G19" s="1" t="n">
         <v>500</v>
@@ -950,14 +990,17 @@
       <c r="B20" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="1" t="n">
+      <c r="C20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="1" t="n">
         <v>0.272538</v>
       </c>
-      <c r="D20" s="1" t="n">
+      <c r="E20" s="1" t="n">
         <v>183.46</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G20" s="1" t="n">
         <v>50</v>
@@ -974,14 +1017,17 @@
       <c r="B21" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="5" t="n">
         <v>0.264998</v>
       </c>
-      <c r="D21" s="1" t="n">
+      <c r="E21" s="1" t="n">
         <v>188.68</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G21" s="1" t="n">
         <v>50</v>
@@ -996,16 +1042,19 @@
         <v>45793</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="1" t="n">
         <v>0.6854</v>
       </c>
-      <c r="D22" s="1" t="n">
+      <c r="E22" s="1" t="n">
         <v>72.95</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G22" s="1" t="n">
         <v>50</v>
@@ -1044,7 +1093,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1837,7 +1886,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>35</v>
@@ -1853,9 +1902,7 @@
       <c r="C2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="G2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
@@ -1867,10 +1914,7 @@
       <c r="C3" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="1" t="n">
-        <f aca="false">SUM(B2:B1000)</f>
-        <v>86.61</v>
-      </c>
+      <c r="G3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
@@ -1913,7 +1957,7 @@
         <v>7.42</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1946,7 +1990,7 @@
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.21"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.53"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.43"/>
@@ -1958,28 +2002,28 @@
         <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1987,19 +2031,19 @@
         <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="E2" s="6" t="n">
-        <v>52110</v>
+        <v>45565</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H2" s="1" t="n">
         <v>2500</v>
@@ -2010,19 +2054,19 @@
         <v>31</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>47088</v>
+        <v>47118</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H3" s="1" t="n">
         <v>500</v>
@@ -2033,16 +2077,19 @@
         <v>34</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>53</v>
+      <c r="E4" s="7" t="n">
+        <v>47118</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H4" s="1" t="n">
         <v>1000</v>
@@ -2053,19 +2100,19 @@
         <v>32</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>47695</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H5" s="1" t="n">
         <v>1000</v>

</xml_diff>